<commit_message>
mise a jour notes.py
</commit_message>
<xml_diff>
--- a/data/CENTRE_PAR_DEFAUT/candidats.xlsx
+++ b/data/CENTRE_PAR_DEFAUT/candidats.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>N° Table</t>
   </si>
@@ -29,30 +29,6 @@
   </si>
   <si>
     <t>Ecole de provenance</t>
-  </si>
-  <si>
-    <t>KOUGBADJI</t>
-  </si>
-  <si>
-    <t>SOMALON</t>
-  </si>
-  <si>
-    <t>David</t>
-  </si>
-  <si>
-    <t>Elise</t>
-  </si>
-  <si>
-    <t>Masculin</t>
-  </si>
-  <si>
-    <t>Féminin</t>
-  </si>
-  <si>
-    <t>Djigangnonhou</t>
-  </si>
-  <si>
-    <t>Doko</t>
   </si>
 </sst>
 </file>
@@ -384,7 +360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -404,40 +380,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>1234</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3">
-        <v>1235</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>